<commit_message>
BBQ EN: ronda de la revisión final regenerada (4 entregables), gates G1-G9 VERDE, F2-NOTAS §9 y sha256 de §8
Ninguna cifra del caso cambia (solo el texto de consumibles_pct, 4% → 3.5%); landing con «the example in the
Word plan» (comillas simples del TS; esbuild OK).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Via: Claude Code
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/bbq-catering-business-plan/bbq-catering-financial-projections.xlsx
+++ b/astro-site/public/dl/bbq-catering-business-plan/bbq-catering-financial-projections.xlsx
@@ -1729,7 +1729,7 @@
       </c>
       <c r="D7" s="28" t="inlineStr">
         <is>
-          <t>A new offset or reverse-flow smoker trailer, 500-gallon class (wood, charcoal or pellets). Examples we read: Meadow Creek TS500 at $20,395 (webstaurantstore.com); Yoder Frontiersman at $8,495-$16,295 plus shipping (yodersmokers.com). The tow vehicle is YOUR pickup, at 0 in this plan. If you don't have one, budget a used pickup that tows at least 3,000 lb (1,360 kg): roughly 25,000-40,000 (Kit estimate).</t>
+          <t>A new offset or reverse-flow smoker trailer, 500-gallon class (wood, charcoal or pellets). Examples we read: Meadow Creek TS500 at $20,395 (webstaurantstore.com); Yoder Frontiersman at $8,495-$16,295 plus shipping (yodersmokers.com). The tow vehicle is YOUR pickup, at 0 in this plan. If you don't have one, budget a used pickup that tows at least 5,000 lb (2,270 kg), checked against the loaded trailer weight: roughly 25,000-40,000 (Kit estimate).</t>
         </is>
       </c>
       <c r="E7" s="31" t="inlineStr">
@@ -5558,7 +5558,7 @@
       </c>
       <c r="J19" s="35" t="inlineStr">
         <is>
-          <t>Average number of people working each event: about 1.5 on a drop-off, 3 on a staffed buffet, 4 on a full-service company event, 5 at a wedding and 4 on a live-fire booking (Kit estimate). Raise it for bigger events: the staffing sizes itself.</t>
+          <t>Average number of people working each event: about 1.5 on a drop-off, 3 on a staffed buffet for 70, 5 on a full-service company event, 7 at a wedding with the live pit (2 on the pit and 5 servers, as in the calculator's example) and 5 on a live-fire booking (Kit estimate). Weighted by the example mix in the Word plan, that averages about 3.4. Raise it for bigger events: the staffing sizes itself.</t>
         </is>
       </c>
     </row>
@@ -6566,7 +6566,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="45" customHeight="1">
+    <row r="59" ht="59.75" customHeight="1">
       <c r="A59" t="inlineStr">
         <is>
           <t>Smoker yield</t>
@@ -6584,7 +6584,7 @@
       </c>
       <c r="D59" s="17" t="inlineStr">
         <is>
-          <t>Brisket and pork butt lose about half their weight in the smoker: 300 guests need roughly 200 lb (91 kg) of raw meat. Buy and cost by raw weight.</t>
+          <t>Brisket and pork butt lose about half their weight in the smoker: 300 guests need roughly 200 lb (91 kg) of raw meat at 1/3 lb cooked per guest; at the calculator's 8 oz, about 270 lb (123 kg). Buy and cost by raw weight.</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D64" s="17" t="inlineStr">
         <is>
-          <t>Median hourly wages for restaurant cooks (35-2014), nonrestaurant food servers (35-3041) and chefs and head cooks (35-1011); 75th percentile $21.45 for cooks and $18.51 for servers. The plan pays the pit cook near the 75th percentile and the owner/pitmaster below the chefs and head cooks median: the rest comes from profit.</t>
+          <t>Mean hourly wages for restaurant cooks (35-2014) and nonrestaurant food servers (35-3041), and the median for chefs and head cooks (35-1011); 75th percentile $21.45 for cooks and $18.51 for servers. The plan pays the pit cook near the 75th percentile and the owner/pitmaster below the chefs and head cooks median: the rest comes from profit.</t>
         </is>
       </c>
     </row>

</xml_diff>